<commit_message>
disable keams enable embed
</commit_message>
<xml_diff>
--- a/data/分群結果.xlsx
+++ b/data/分群結果.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C162"/>
+  <dimension ref="A1:C194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,7 +435,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -450,7 +450,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -465,7 +465,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -480,7 +480,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -495,7 +495,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -525,7 +525,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -540,7 +540,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -600,7 +600,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -615,7 +615,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -705,7 +705,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -735,7 +735,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -840,7 +840,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -885,7 +885,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1005,7 +1005,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1020,7 +1020,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1110,7 +1110,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1230,7 +1230,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -1320,7 +1320,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -1380,7 +1380,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -1470,7 +1470,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -1590,7 +1590,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -1620,7 +1620,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -1665,7 +1665,7 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -1680,7 +1680,7 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -1710,7 +1710,7 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -1785,7 +1785,7 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -1815,7 +1815,7 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -1875,7 +1875,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -1965,7 +1965,7 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -1980,7 +1980,7 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -2025,7 +2025,7 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -2070,7 +2070,7 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -2115,7 +2115,7 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -2145,7 +2145,7 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -2160,7 +2160,7 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -2175,7 +2175,7 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -2220,7 +2220,7 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -2250,7 +2250,7 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -2265,7 +2265,7 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -2295,7 +2295,7 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -2355,7 +2355,7 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -2370,7 +2370,7 @@
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -2385,7 +2385,7 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -2415,7 +2415,7 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -2430,7 +2430,7 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -2445,7 +2445,7 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -2475,7 +2475,7 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -2490,7 +2490,7 @@
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -2505,7 +2505,7 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -2535,7 +2535,7 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -2565,7 +2565,7 @@
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -2580,7 +2580,7 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -2595,7 +2595,7 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -2604,13 +2604,13 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>utg under_the_gun 槍口位 大盲注 左手 邊 第一 個 槍口位 翻牌前 最先 行動 德州撲克 裡 位置 越靠後越 有利 因此 坐在 槍口位 玩家 最 動 玩家 起 手牌 要求 比 其他 位置 要 高 往往 翻牌前 棄牌</t>
+          <t>utg under_the_gun 槍口位 大盲注 左手 邊 第一 個 槍口位 翻牌前 最先 行動 德州撲克 裡 位置 越靠後越 有利 因此 坐在 槍口位 玩家 最 動 玩家 起手牌 要求 比 其他 位置 要 高 往往 翻牌前 棄牌</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -2625,7 +2625,7 @@
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -2670,7 +2670,7 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -2685,7 +2685,7 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -2700,7 +2700,7 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -2715,7 +2715,7 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -2775,7 +2775,7 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -2845,6 +2845,486 @@
       <c r="C162" t="inlineStr">
         <is>
           <t>每個 玩家 遊戲 樹 任何 決策點 帶 著 一手 牌 範圍 當你 特定 位置 特定 手牌 有 一 張牌 你 對手 範圍 相關 時 那 張牌 認為 阻擋牌 它 之所以 稱 阻擋牌 因為 它 讓 你 對手 更 有 可能 或 更 不 可能 持有 某種 牌</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>4</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>開局加注該下多少？常見的標準開局加注是 2 到 3 個大盲(BB)。線上多用 2~2.5 BB，實體現場多用 3 BB。若前面已有人只跟大盲(limp)進場，通常每多一個 limper 就多加 1 BB。</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>開局 加注 該下 多少 ？ 常見 標準 開局 加注 2 到 3 個大盲 bb 線上 多用 2 ~ 2.5 bb 實體 現場 多用 3 bb 前面 已有 人 只 跟 大盲 limp 進場 通常 每多 limper 多加 1 bb</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>0</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>持續下注(c_bet)要下多大？翻牌後第一槍通常下底池的三分之一到三分之二。對手不容易聽牌可以下小，約 1/3 底池；很多同花、順子聽牌就下大一點，約 2/3 到 3/4 底池施壓。</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>持續下注 c_bet 要 下 多 大 ？ 翻牌後 第一 槍 通常 下底 池 三分之一 到 三分之二 對手 不 容易 聽牌 可以 下 小 約 1 3 底池 很多 同花 順子 聽牌 下 大 一點 約 2 3 到 3 4 底池 施壓</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>1</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>下注大小要用「底池的幾分之幾」來想，而不是固定幾個籌碼。用相對底池的概念，才能在不同底池大小下都做出合理的下注。</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>下注 大小 要 用 底池 幾分 之 幾 來 想 不是 固定 幾個 籌碼 用 相 底池 概念 才能 不同 底池 大小 下 做出 合理 下注</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>4</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>翻牌前再加注(3bet)該下多少？面對對手的開局加注，新手可以簡化成原加注額的 3 到 4 倍。位置好可下小一點，位置差(在對手前面行動)就下大一點來保護。</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>翻牌前 再 加注 3bet 該下 多少 ？ 面對 對手 開局 加注 新手 可以 簡 化成 原 加注 額 3 到 4 倍 位置 好 可下 小 一點 位置 差 對手 前面 行動 下 大 一點 來 保護</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>0</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>新手常見的下注尺寸錯誤：價值大牌時下很大、詐唬時下很小，這會讓觀察力好的對手一眼看穿你的牌力。應該讓相同情境下的下注大小盡量一致。</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>新手 常見 下注 尺寸 錯誤 價值 大牌 時下 很大 詐唬 時下 很小 這會 讓 觀察力 好 對手 一眼看穿 你 牌力 應該 讓 相同 情境 下 下注 大小 盡量 一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>0</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>下注太小的問題：在大底池只下一點點，等於送給對手很好的賠率去追聽牌。想要保護成手牌或施壓，就要下到足夠的大小。</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>下注 太小 問題 大底 池 只 下 一點點 等於 送給 對手 很 好 賠率 去 追 聽牌 想要 保護成 手牌 或 施壓 就要 下到 足夠 大小</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>0</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>什麼是價值下注？價值下注是指你覺得自己的手牌是領先的，因此下注是為了從對手那裡「榨取更多籌碼」，下注金額不能太大，否則會嚇跑對手</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>什麼 價值 下注 ？ 價值 下注 你 覺得 自己 手牌 領先 因此 下注 從 對手 那裡 榨取 更多 籌碼 下注 金額 不能 太 大 否則 會嚇 跑 對手</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>0</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>下注是你在遊戲中唯一能主動發聲的方式，所以才會有這麼多種下注策略。每一種下注金額、時機、方式，其實都是在告訴對手一個訊息，也是在試圖引導他們做出你希望的反應。不同情況，需要不同目的的下注，增加不可預測性，讓對手無法掌握你的節奏</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>下注 你 遊戲 中 唯一 能主動 發聲 方式 所以 才 有 這麼 多種 下注 策略 每一種 下注 金額 時機 方式 其實 告訴 對手 訊息 試圖 引導 他們 做出 你 希望 反應 不 同情 況 需要 不同 目的 下注 增加 不可 預測性 讓 對手 無法 掌握 你 節奏</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>1</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>輪到你才行動。在還沒輪到你的時候就先表態、先亮牌或先把牌丟出去，會洩漏資訊、影響其他玩家的決定，是牌桌上的大忌。</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>你 才 行動 還沒輪 到 你 時候 先表態 先 亮牌 或 先 牌 丟 出去 會洩漏 資訊 影響 其他 玩家 決定 牌 桌上 大忌</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>4</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>下注時請一次把籌碼放到下注線前，不要分好幾次把籌碼一點一點推出去，分次推注通常不被允許，只會算第一次的金額。</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>下注 時請 一次 籌碼 放到 下注 線前 不要 分好 幾次 籌碼 一點 一點 推出 去 分 次 推注 通常 不 允許 只會算 第一次 金額</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>0</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>還沒攤牌前，不要評論正在進行的這手牌，也不要把你已蓋掉的牌內容說出來。討論進行中的牌局會影響仍在牌局裡的玩家，屬於違規行為。</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>還沒攤 牌前 不要 評論 正在 進行 這手牌 不要 你 已 蓋 掉 牌 內容 說 出來 討論 進行 中 牌局 影響 仍 牌局 裡的 玩家 屬 違規行</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>1</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>保護好你的底牌：用一個籌碼或專用牌蓋壓在牌上，避免荷官誤收或和別人的棄牌混在一起。一旦底牌碰到棄牌堆，這手牌通常就作廢了。</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>保護 好 你 底牌 用 籌碼 或 專用 牌蓋壓 牌 上 避免 荷官 誤收 或 和 別人 棄牌 混在 一起 一旦 底牌 碰到 棄牌 堆 這手牌 通常 就作 廢</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>1</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>不要對其他玩家的打法指指點點或當場教學，也不要催促別人快點行動。給每位玩家合理的思考時間，是基本的尊重。</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>不要 其他 玩家 打法 指指 點點 或 當場 教學 不要 催促 別人 快點 行動 給 每位 玩家 合理 思考 時間 基本 尊重</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>0</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>該帶多少錢上桌？現金桌只帶你「願意輸掉」的金額，絕對不要帶上全部身家或生活費。把撲克的資金和日常生活開銷完全分開。</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>該 帶 多少 錢 上桌 ？ 現金桌 只 帶 你 願意 輸掉 金額 絕對 不要 帶上 全部 身家 或 生活 費 撲克 資金 和 日常生活 開銷 完全 分開</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>0</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>資金管理的常見原則：玩現金桌時，準備約 20 到 30 個買入的總資金，這樣即使連續輸幾局，也不會一次就破產出局。</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>資金 管理 常見 原則 玩現 金桌 時 準備 約 20 到 30 個 買入 總資金 這樣 即使 連續 輸幾局 不會 一次 破產 出局</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>0</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>選擇適合自己資金的盲注級別，不要越級挑戰高盲注的桌。級別越高、對手越強、波動越大，新手應該從小級別開始累積經驗與資金。</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>選擇 適合 自己 資金 盲注 級別 不要 越級 挑戰高 盲注 桌 級別 越 高 對手 越強 波動 越大 新手 應該 從 小級別 開始 累積 經驗 資金</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>0</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>設定停損點：給自己定一個「今天輸到多少就離桌」的金額。輸牌後容易情緒化追損(上頭)，事先設好停損能保護你的資金與心態。</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>設定 停 損點 給 自己 定一個 今天 輸到 多少 離桌 金額 輸牌 後 容易 情緒化 追損 上頭 事先 設好 停 損能 保護 你 資金 心態</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>0</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>錦標賽的資金需求比現金桌更高。因為錦標賽名次波動(方差)很大，常常要打很多場才會中獎，建議單場買入只占總資金更小的比例。</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>錦標賽 資金 需求 比現 金桌 更 高 因為 錦 標賽 名次 波動 方差 很大 常常 要 打 很多 場才會 中獎 建議 單場 買入 只 占 總資金 更 小 比例</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>4</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>哪些起手牌一定能玩？大對子 AA、KK、QQ、JJ，以及 AK、AQ 這類強牌，在任何位置幾乎都可以加注進場，是新手最安全的選擇。</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>哪些 起手牌 一定 能 玩 ？ 大 對子 aa kk qq jj ak aq 這類 強牌 任何 位置 幾乎 可以 加注 進場 新手 最 安全 選擇</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>0</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>新手可以玩的中等起手牌：中小對子(例如 99、88、77)、同花的 A(如 A5s)、以及同花連張(如 JTs、98s)。這些牌有成順子或同花的潛力。</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>新手 可以 玩 中等 起手牌 中 小對子 例如 99 88 77 同花 a 如 a5s 同花 連張 如 jts 98s 牌 有 成 順子 或 同花 潛力</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>3</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>該直接丟掉的起手牌：不成對、又不同花、數字又差很多的雜牌，新手直接棄牌就好，不要因為想玩而勉強進場。</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>該 直接 丟掉 起手牌 不成 又 不同 花 數字 又 差 很多 雜牌 新手 直接 棄牌 好 不要 因為 想 玩 勉強 進場</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>1</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>位置會大幅影響起手牌選擇：在前面位置(如槍口位 UTG)後面還有很多人沒行動，只玩很強的牌；在後面位置(如按鈕位 BTN)可以玩寬一點。口訣是「位置越好，能玩的牌越多」。</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>位置 大幅 影響 起手牌 選擇 前面 位置 如 槍口位 utg 後 面 還有 很多 人 沒 行動 只 玩 很強 牌 在後面 位置 如 按鈕位 btn 可以 玩 寬 一點 口訣 位置 越 好 能 玩 牌 越 多</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>0</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>同花不代表什麼牌都能玩。雖然同花的兩張牌比不同花稍強一點點，但像 92 同花這種差距太大的牌還是該丟，別被「同花」兩個字騙了。</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>同花 不 代表 什麼 牌 能 玩 雖然 同花 兩 張牌 比 不同 花 稍強 一點點 但 像 92 同花 這種 差距 太大 牌 還是 該 丟 別 同花 兩個 字 騙</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>4</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>該不該 limp(只跟大盲、不加注就進場)？新手通常不建議 limp，因為放棄了主動權、也容易讓很多人一起看翻牌。要玩這手牌就用加注進場，不想玩就棄牌。</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>該 不 該 limp 只 跟 大盲 不 加注 進場 ？ 新手 通常 不建議 limp 因為 放棄 主動權 容易 讓 很多 人 一起 看 翻牌 要 玩 這手牌 用 加注 進場 不想 玩 棄牌</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>1</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>人少的牌桌(例如 6 人桌)起手牌可以比 9 人滿桌玩得更寬，因為位置輪轉快、盲注壓力大；滿桌則要打得更緊一些。</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>人少 牌桌 例如 6 人桌 起手牌 可以 比 9 人滿 桌玩得 更 寬 因為 位置 輪 轉快 盲注 壓力 大 滿桌則 要 打 得 更 緊 一些</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>3</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>最常見的新手錯誤是「玩太多手牌」。覺得每手都想參與，結果常拿著弱牌進場、翻牌後陷入兩難。正確做法是打緊一點，多數爛牌直接棄掉。</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>最常見 新手 錯誤 玩太多 手牌 覺得 每手 想 參 結果 常拿著 弱牌 進場 翻牌後 陷入 兩難 正確 做法 打緊 一點 多數爛牌 直接 棄掉</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>4</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>新手很愛 limp(只跟不加注)進場。這會放棄主動權、把底池搞得很多人一起玩。建議：值得玩的牌就用加注進場，不值得就棄牌，少用 limp。</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>新手 很 愛 limp 只 跟 不 加注 進場 這會 放棄 主動權 底池 搞 得 很多 人 一起 玩 建議 值得 玩 牌 用 加注 進場 不 值得 棄牌 少 用 limp</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>0</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>無腦跟注是燒錢的壞習慣：沒有明確理由就一直跟注到底。每次跟注前先問自己「我跟的理由是什麼」，要嘛有勝算或好賠率，要嘛就棄牌。</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>無腦 跟注 燒錢 壞 習慣 沒有 明確 理由 一直 跟注 到底 每次 跟注 前先問 自己 我 跟 理由 什麼 要 嘛 有 勝算 或 好 賠率 要 嘛 棄牌</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>0</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>追聽牌不算賠率：為了湊同花或順子一路跟注，卻沒算底池賠率划不划算。聽牌要看「補牌張數」和「底池給的賠率」是否值得追。</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>追聽牌 不算 賠率 湊 同花 或 順子 一路 跟注 卻 沒算 底池賠率 划 不划算 聽牌 要 看 補牌 張數 和 底池給 賠率 是否 值得 追</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>3</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>上頭(tilt)：輸了一手大牌之後情緒失控、開始亂打想討回來，結果輸更多。最好的處理方式是先離桌休息、冷靜下來，再決定要不要繼續。</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>上頭 tilt 輸 一手 大牌 之後情緒 失控 開始 亂 打 想 討 回來 結果 輸 更 多 最好 處理 方式 先離桌 休息 冷靜 下來 再 決定 要 不要 繼續</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>0</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>太黏成手牌：拿到一對 A 就死不放手，明明牌面出現同花或順子的危險、對手又重注，還是硬跟到底。學會在情況不對時放掉好牌，是進步的關鍵。</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>太 黏成 手牌 拿到 一對 a 死 不 放手 明明 牌面 出現 同花 或 順子 危險 對手 又 重注 還是 硬 跟 到底 學會 情況 不 時 放掉 好牌 進步 關鍵</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>1</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>不看位置就行動：忽略自己在這手牌是先行動還是後行動。位置差時要更謹慎，位置好(較晚行動)才有資訊優勢可以玩寬一點。</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>不看 位置 行動 忽略 自己 這手牌 先 行動 還是 後 行動 位置 差時 要 更 謹慎 位置 好 較晚 行動 才 有 資訊 優勢 可以 玩 寬 一點</t>
         </is>
       </c>
     </row>

</xml_diff>